<commit_message>
Complete the human review for Svarah and AESRC
Svarah (60 clips) and AESRC (28 clips) join the TIE sheet, same protocol and
same annotator. Correcting the reference drops mean WER on the reviewed subset
by 7.8 pp on Svarah and 3.1 pp on AESRC, against 47.8 pp on TIE. The AESRC drop
is not significant. The curated corpora are hard because the speech is hard,
while TIE is hard largely because its references are wrong.

All three sheets now share one 15-label vocabulary, so the same cause reads the
same way everywhere. The TIE labels were renamed to match without changing any
clip's classification. Svarah's sheet is renamed to review_sheet.* for
consistency, and the 499-row flagged pool it was sampled from is no longer
tracked.

Half of Svarah's flagged clips fail on number formatting rather than on speech:
models that read a digit string aloud are scored against a reference that
writes digits.
</commit_message>
<xml_diff>
--- a/analysis/tie_validation/review_sheet.xlsx
+++ b/analysis/tie_validation/review_sheet.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="AG2" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH2" s="5" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>25.00</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>25.00</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="AG3" s="5" t="inlineStr">
         <is>
-          <t>Technical vocabulary (jargon, numbers, names)</t>
+          <t>Technical vocabulary</t>
         </is>
       </c>
       <c r="AH3" s="5" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="AG6" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH6" s="5" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.50</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="AG7" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Number formatting</t>
         </is>
       </c>
       <c r="AH7" s="5" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>18.6</t>
+          <t>18.60</t>
         </is>
       </c>
       <c r="S8" s="5" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="AG9" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH9" s="5" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="AG10" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH10" s="5" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>30.3</t>
+          <t>30.30</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="AG11" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH11" s="5" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>38.1</t>
+          <t>38.10</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="AG13" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH13" s="5" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="AG14" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH14" s="5" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="AG15" s="5" t="inlineStr">
         <is>
-          <t>Misalignment (wrong clip boundary)</t>
+          <t>Misalignment</t>
         </is>
       </c>
       <c r="AH15" s="5" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="AG16" s="5" t="inlineStr">
         <is>
-          <t>Misalignment (wrong clip boundary)</t>
+          <t>Misalignment</t>
         </is>
       </c>
       <c r="AH16" s="5" t="inlineStr">
@@ -3515,9 +3515,8 @@
       </c>
       <c r="Z17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">By what is the concentration of Bn⁺ in the solution?
-So, Rₙ⁻Bn⁺ (resin) means activity of Bn⁺ in the resin, and Bn⁺ (S) means activity of Bn⁺ in the solution.
-</t>
+          <t>By what is the concentration of Bn⁺ in the solution?
+So, Rₙ⁻Bn⁺ (resin) means activity of Bn⁺ in the resin, and Bn⁺ (S) means activity of Bn⁺ in the solution.</t>
         </is>
       </c>
       <c r="AA17" s="5" t="inlineStr">
@@ -3552,7 +3551,7 @@
       </c>
       <c r="AG17" s="5" t="inlineStr">
         <is>
-          <t>Misalignment (wrong clip boundary)</t>
+          <t>Misalignment</t>
         </is>
       </c>
       <c r="AH17" s="5" t="inlineStr">
@@ -3736,7 +3735,7 @@
       </c>
       <c r="AG18" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH18" s="5" t="inlineStr">
@@ -4058,13 +4057,12 @@
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">I won't say assumption, but it is an abstraction.
+          <t>I won't say assumption, but it is an abstraction.
 We'll talk about how it affects our analysis.
 As many number of processors as you need, which means it is valid for a single processor machine or even millions of processors.
 Yes.
 Ahmm.
-So, one is the amount of resources, how much memory I have, how much local versus shared.
-</t>
+So, one is the amount of resources, how much memory I have, how much local versus shared.</t>
         </is>
       </c>
       <c r="AA20" s="5" t="inlineStr">
@@ -4206,7 +4204,7 @@
       </c>
       <c r="S21" s="5" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>50.00</t>
         </is>
       </c>
       <c r="T21" s="5" t="inlineStr">
@@ -4278,7 +4276,7 @@
       </c>
       <c r="AG21" s="5" t="inlineStr">
         <is>
-          <t>Technical vocabulary (jargon, numbers, names)</t>
+          <t>Technical vocabulary</t>
         </is>
       </c>
       <c r="AH21" s="5" t="inlineStr"/>
@@ -4366,32 +4364,32 @@
       </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
@@ -4570,7 +4568,7 @@
       </c>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>33.1</t>
+          <t>33.10</t>
         </is>
       </c>
       <c r="V23" s="5" t="inlineStr">
@@ -4631,7 +4629,7 @@
       </c>
       <c r="AG23" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH23" s="5" t="inlineStr">
@@ -4723,32 +4721,32 @@
       </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>35.00</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="R24" s="5" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>27.5</t>
+          <t>27.50</t>
         </is>
       </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>15.50</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
@@ -4925,7 +4923,7 @@
       </c>
       <c r="T25" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U25" s="5" t="inlineStr">
@@ -4991,7 +4989,7 @@
       </c>
       <c r="AG25" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH25" s="5" t="inlineStr">
@@ -5103,7 +5101,7 @@
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
@@ -5281,7 +5279,7 @@
       </c>
       <c r="T27" s="5" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>50.00</t>
         </is>
       </c>
       <c r="U27" s="5" t="inlineStr">
@@ -5440,32 +5438,32 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>24.00</t>
         </is>
       </c>
       <c r="R28" s="5" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>14.4</t>
+          <t>14.40</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
@@ -5619,32 +5617,32 @@
       </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="R29" s="5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="T29" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U29" s="5" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="V29" s="5" t="inlineStr">
@@ -6066,7 +6064,7 @@
       </c>
       <c r="AG31" s="5" t="inlineStr">
         <is>
-          <t>Misalignment (wrong clip boundary)</t>
+          <t>Misalignment</t>
         </is>
       </c>
       <c r="AH31" s="5" t="inlineStr">
@@ -6158,32 +6156,32 @@
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.50</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>25.00</t>
         </is>
       </c>
       <c r="R32" s="5" t="inlineStr">
         <is>
-          <t>37.5</t>
+          <t>37.50</t>
         </is>
       </c>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>25.00</t>
         </is>
       </c>
       <c r="T32" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>20.00</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
@@ -6243,7 +6241,7 @@
       </c>
       <c r="AG32" s="5" t="inlineStr">
         <is>
-          <t>Misalignment (wrong clip boundary)</t>
+          <t>Misalignment</t>
         </is>
       </c>
       <c r="AH32" s="5" t="inlineStr">
@@ -6355,7 +6353,7 @@
       </c>
       <c r="T33" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U33" s="5" t="inlineStr">
@@ -6540,7 +6538,7 @@
       </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>15.9</t>
+          <t>15.89</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
@@ -6705,7 +6703,7 @@
       </c>
       <c r="R35" s="5" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="S35" s="5" t="inlineStr">
@@ -6715,7 +6713,7 @@
       </c>
       <c r="T35" s="5" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="U35" s="5" t="inlineStr">
@@ -6880,22 +6878,22 @@
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>50.00</t>
         </is>
       </c>
       <c r="R36" s="5" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.50</t>
         </is>
       </c>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.50</t>
         </is>
       </c>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>25.00</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
@@ -6925,8 +6923,7 @@
       </c>
       <c r="Z36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Example, for hollow shaft, we can see that this comes out to be equal to Td₀/2, and Iₚ will be...
-</t>
+          <t>Example, for hollow shaft, we can see that this comes out to be equal to Td₀/2, and Iₚ will be...</t>
         </is>
       </c>
       <c r="AA36" s="5" t="inlineStr">
@@ -7140,7 +7137,7 @@
       </c>
       <c r="AG37" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names), Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Technical vocabulary, Disfluency</t>
         </is>
       </c>
       <c r="AH37" s="5" t="inlineStr">
@@ -7498,7 +7495,7 @@
       </c>
       <c r="AG39" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Disfluency (fillers, repetitions, false starts)</t>
+          <t>Reference error, Disfluency</t>
         </is>
       </c>
       <c r="AH39" s="5" t="inlineStr">
@@ -7680,7 +7677,7 @@
       </c>
       <c r="AG40" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH40" s="5" t="inlineStr">
@@ -7792,7 +7789,7 @@
       </c>
       <c r="T41" s="5" t="inlineStr">
         <is>
-          <t>12.7</t>
+          <t>12.70</t>
         </is>
       </c>
       <c r="U41" s="5" t="inlineStr">
@@ -7953,7 +7950,7 @@
       </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>12.90</t>
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr">
@@ -7973,7 +7970,7 @@
       </c>
       <c r="T42" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U42" s="5" t="inlineStr">
@@ -8147,7 +8144,7 @@
       </c>
       <c r="S43" s="5" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="T43" s="5" t="inlineStr">
@@ -8221,7 +8218,7 @@
       </c>
       <c r="AG43" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH43" s="5" t="inlineStr">
@@ -8401,7 +8398,7 @@
       </c>
       <c r="AG44" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH44" s="5" t="inlineStr">
@@ -8493,32 +8490,32 @@
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="Q45" s="5" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="R45" s="5" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>22.00</t>
         </is>
       </c>
       <c r="S45" s="5" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>32.00</t>
         </is>
       </c>
       <c r="T45" s="5" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="U45" s="5" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>13.60</t>
         </is>
       </c>
       <c r="V45" s="5" t="inlineStr">
@@ -8580,7 +8577,7 @@
       </c>
       <c r="AG45" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH45" s="5" t="inlineStr">
@@ -8762,7 +8759,7 @@
       </c>
       <c r="AG46" s="5" t="inlineStr">
         <is>
-          <t>Reference error, Technical vocabulary (jargon, numbers, names)</t>
+          <t>Reference error, Technical vocabulary</t>
         </is>
       </c>
       <c r="AH46" s="5" t="inlineStr">

</xml_diff>